<commit_message>
Fix identity leak in PRISMA checklist read-me notes
</commit_message>
<xml_diff>
--- a/07_prisma_2020_checklist.xlsx
+++ b/07_prisma_2020_checklist.xlsx
@@ -522,7 +522,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>The 27 items of the PRISMA 2020 Statement (Page et al., 2021), item by item, mapped to where the article addresses each one (section/spreadsheet) or flagged as not applicable, not done, or pending completion by Samuel (funding, competing interests, public protocol registration — information this repository does not have).</t>
+          <t>The 27 items of the PRISMA 2020 Statement (Page et al., 2021), item by item, mapped to where the article addresses each one (section/spreadsheet) or flagged as not applicable, not done, or pending completion by the authors (funding, competing interests, public protocol registration — information this repository does not have).</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Addressed = the article covers the item. Partial = covers it in part, with the caveat in the "Note" column. Not applicable = the item does not apply to this review design (e.g. effect meta-analysis, which this SLR does not do). Not done = the item would in principle apply, but was not carried out (disclosed here, not hidden — the same transparency logic already used for the below-threshold kappa). Pending — to be completed = information that only Samuel has is missing.</t>
+          <t>Addressed = the article covers the item. Partial = covers it in part, with the caveat in the "Note" column. Not applicable = the item does not apply to this review design (e.g. effect meta-analysis, which this SLR does not do). Not done = the item would in principle apply, but was not carried out (disclosed here, not hidden — the same transparency logic already used for the below-threshold kappa). Pending — to be completed = information that only the authors have is missing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stale section-number references in kappa worksheet and PRISMA checklist
</commit_message>
<xml_diff>
--- a/07_prisma_2020_checklist.xlsx
+++ b/07_prisma_2020_checklist.xlsx
@@ -757,7 +757,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.3 Eligibility Criteria</t>
+          <t>Method, 3.3 Eligibility Criteria</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
@@ -785,7 +785,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.2 Search Strategy; see also the "01_search_strategy_by_database.xlsx" spreadsheet</t>
+          <t>Method, 3.2 Search Strategy; see also the "01_search_strategy_by_database.xlsx" spreadsheet</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr"/>
@@ -813,7 +813,7 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.2 (full strings) + "01_search_strategy_by_database.xlsx"</t>
+          <t>Method, 3.2 (full strings) + "01_search_strategy_by_database.xlsx"</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr"/>
@@ -841,7 +841,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.5-2.7 (two independent raters) + 2.11 Use of Artificial Intelligence (automation tools disclosed)</t>
+          <t>Method, 3.5-3.7 (two independent raters) + 3.11 Use of Artificial Intelligence (automation tools disclosed)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr"/>
@@ -869,7 +869,7 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.9 Data Extraction</t>
+          <t>Method, 3.9 Data Extraction</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr"/>
@@ -897,7 +897,7 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.9 (table of the 13 extraction fields — adaptation: thematic SLR, not intervention-effect review)</t>
+          <t>Method, 3.9 (table of the 13 extraction fields — adaptation: thematic SLR, not intervention-effect review)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
@@ -925,7 +925,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.9 (same table)</t>
+          <t>Method, 3.9 (same table)</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr"/>
@@ -953,7 +953,7 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.7 Quality Assessment (Q4-Q8) — a purpose-built instrument, not a named standardized tool (e.g. Newcastle-Ottawa)</t>
+          <t>Method, 3.7 Quality Assessment (Q4-Q8) — a purpose-built instrument, not a named standardized tool (e.g. Newcastle-Ottawa)</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr"/>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.12 Synthesis and Analysis (all 83 included studies enter the 5 dimensions)</t>
+          <t>Method, 3.12 Synthesis and Analysis (all 83 included studies enter the 5 dimensions)</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr"/>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.10 Thematic Coding (codebook)</t>
+          <t>Method, 3.10 Thematic Coding (codebook)</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.12 (counts + narrative synthesis per dimension)</t>
+          <t>Method, 3.12 (counts + narrative synthesis per dimension)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr"/>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Discussion, 4.2 (review of the 65 Q8 decomposition cases, 17 downgrades/8 upgrades)</t>
+          <t>Discussion, 5.2 (review of the 65 Q8 decomposition cases, 17 downgrades/8 upgrades)</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.5 Selection Process (table) + "artigo/imagens/2.5_flow-selection-prisma_en.pdf" (not yet inserted into the body of the article)</t>
+          <t>Method, 3.5 Selection Process (table) + "artigo/imagens/2.5_flow-selection-prisma_en.pdf" (not yet inserted into the body of the article)</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Results, 3.1 Corpus Characterization + "05_data_extraction_83_included.xlsx" + Appendix A (list of the 83)</t>
+          <t>Results, 4.1 Corpus Characterization + "05_data_extraction_83_included.xlsx" + Appendix A (list of the 83)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr"/>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>"05_data_extraction_83_included.xlsx" + cited exemplars (Results, 3.3-3.5) — adaptation: narrative findings, not effect estimates</t>
+          <t>"05_data_extraction_83_included.xlsx" + cited exemplars (Results, 4.3-4.5) — adaptation: narrative findings, not effect estimates</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr"/>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Results, 3.1-3.5</t>
+          <t>Results, 4.1-4.5</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr"/>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Results, 3.2-3.5 (counts and percentages per dimension)</t>
+          <t>Results, 4.2-4.5 (counts and percentages per dimension)</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Discussion, 4.2</t>
+          <t>Discussion, 5.2</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Discussion, 4.1-4.2</t>
+          <t>Discussion, 5.1-5.2</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr"/>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Discussion (scattered) — see also 4.3 Study Limitations</t>
+          <t>Discussion (scattered) — see also 5.3 Study Limitations</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -1625,7 +1625,7 @@
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Discussion, 4.3 Study Limitations (kappa below threshold, lighter treatment of Research Method and exemplars, item discarded on suspected error)</t>
+          <t>Discussion, 5.3 Study Limitations (kappa below threshold, lighter treatment of Research Method and exemplars, item discarded on suspected error)</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr"/>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>The Discussion ends at the transferability axis (4.2); an explicit section on practical/policy implications for the Judiciary and a future-research agenda is still needed.</t>
+          <t>The Discussion ends at the transferability axis (5.2); an explicit section on practical/policy implications for the Judiciary and a future-research agenda is still needed.</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1685,7 @@
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.1 Study Design (protocol managed in the Parsif.al tool)</t>
+          <t>Method, 3.1 Study Design (protocol managed in the Parsif.al tool)</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Method, 2.4 Protocol Revision (Q1-Q3/Q4-Q8 reclassification; removal of IAM from scope)</t>
+          <t>Method, 3.4 Protocol Revision (Q1-Q3/Q4-Q8 reclassification; removal of IAM from scope)</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr"/>

</xml_diff>